<commit_message>
Resultados de análisis problema4 (1M iteraciones)
</commit_message>
<xml_diff>
--- a/Nuevos DeepWins/Problem4_Bullseye5/Res/Comparativa_12_Neuronas.xlsx
+++ b/Nuevos DeepWins/Problem4_Bullseye5/Res/Comparativa_12_Neuronas.xlsx
@@ -581,43 +581,35 @@
         <v>0.1</v>
       </c>
       <c r="B2" t="n">
-        <v>0.181897</v>
+        <v>0.239735</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1790732034</v>
+        <v>1790732086</v>
       </c>
       <c r="E2" t="n">
-        <v>52</v>
+        <v>170</v>
       </c>
       <c r="F2" t="n">
         <v>200000</v>
       </c>
-      <c r="G2" t="n">
-        <v>0.5836789999999999</v>
-      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>0.661442</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.620132</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="n">
-        <v>0.181047</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0.60221</v>
-      </c>
+        <v>0.24501</v>
+      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
-        <v>0.641176</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.6210830000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M2" t="inlineStr"/>
       <c r="N2" t="n">
         <v>0.2</v>
       </c>
@@ -652,23 +644,23 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732034_18.txt</t>
+          <t>_2_3_3_3_3_1_1790732086_7.txt</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z2" t="n">
         <v>12</v>
       </c>
       <c r="AA2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -682,35 +674,43 @@
         <v>0.1</v>
       </c>
       <c r="B3" t="n">
-        <v>0.239747</v>
+        <v>0.184394</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1790732086</v>
+        <v>1790732034</v>
       </c>
       <c r="E3" t="n">
-        <v>170</v>
+        <v>52</v>
       </c>
       <c r="F3" t="n">
         <v>200000</v>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>0.610015</v>
+      </c>
       <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="inlineStr"/>
+        <v>0.630094</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.619892</v>
+      </c>
       <c r="J3" t="n">
-        <v>0.245023</v>
-      </c>
-      <c r="K3" t="inlineStr"/>
+        <v>0.184358</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.614907</v>
+      </c>
       <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="inlineStr"/>
+        <v>0.582353</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.598187</v>
+      </c>
       <c r="N3" t="n">
         <v>0.2</v>
       </c>
@@ -745,23 +745,23 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732086_10.txt</t>
+          <t>_2_12_1_1790732034_16.txt</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z3" t="n">
         <v>12</v>
       </c>
       <c r="AA3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
@@ -775,7 +775,7 @@
         <v>0.1</v>
       </c>
       <c r="B4" t="n">
-        <v>0.236779</v>
+        <v>0.239733</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -797,7 +797,7 @@
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="n">
-        <v>0.242342</v>
+        <v>0.245085</v>
       </c>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
@@ -838,7 +838,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732086_9.txt</t>
+          <t>_2_3_3_3_3_1_1790732086_14.txt</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -868,7 +868,7 @@
         <v>0.1</v>
       </c>
       <c r="B5" t="n">
-        <v>0.175663</v>
+        <v>0.183638</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -885,25 +885,25 @@
         <v>200000</v>
       </c>
       <c r="G5" t="n">
-        <v>0.616864</v>
+        <v>0.5625</v>
       </c>
       <c r="H5" t="n">
-        <v>0.653605</v>
+        <v>0.648903</v>
       </c>
       <c r="I5" t="n">
-        <v>0.634703</v>
+        <v>0.60262</v>
       </c>
       <c r="J5" t="n">
-        <v>0.17518</v>
+        <v>0.180978</v>
       </c>
       <c r="K5" t="n">
-        <v>0.631579</v>
+        <v>0.590164</v>
       </c>
       <c r="L5" t="n">
         <v>0.635294</v>
       </c>
       <c r="M5" t="n">
-        <v>0.633431</v>
+        <v>0.6118980000000001</v>
       </c>
       <c r="N5" t="n">
         <v>0.2</v>
@@ -939,7 +939,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732034_6.txt</t>
+          <t>_2_12_1_1790732034_4.txt</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
@@ -969,43 +969,35 @@
         <v>0.1</v>
       </c>
       <c r="B6" t="n">
-        <v>0.178623</v>
+        <v>0.239693</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1790732034</v>
+        <v>1790732086</v>
       </c>
       <c r="E6" t="n">
-        <v>52</v>
+        <v>170</v>
       </c>
       <c r="F6" t="n">
         <v>200000</v>
       </c>
-      <c r="G6" t="n">
-        <v>0.600293</v>
-      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>0.642633</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.620742</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="n">
-        <v>0.181897</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0.616279</v>
-      </c>
+        <v>0.244958</v>
+      </c>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
-        <v>0.623529</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0.619883</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
         <v>0.2</v>
       </c>
@@ -1040,23 +1032,23 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732034_3.txt</t>
+          <t>_2_3_3_3_3_1_1790732086_0.txt</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z6" t="n">
         <v>12</v>
       </c>
       <c r="AA6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -1070,7 +1062,7 @@
         <v>0.1</v>
       </c>
       <c r="B7" t="n">
-        <v>0.180623</v>
+        <v>0.181897</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1087,25 +1079,25 @@
         <v>200000</v>
       </c>
       <c r="G7" t="n">
-        <v>0.583573</v>
+        <v>0.5836789999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>0.634796</v>
+        <v>0.661442</v>
       </c>
       <c r="I7" t="n">
-        <v>0.608108</v>
+        <v>0.620132</v>
       </c>
       <c r="J7" t="n">
-        <v>0.180828</v>
+        <v>0.181047</v>
       </c>
       <c r="K7" t="n">
-        <v>0.587879</v>
+        <v>0.60221</v>
       </c>
       <c r="L7" t="n">
-        <v>0.570588</v>
+        <v>0.641176</v>
       </c>
       <c r="M7" t="n">
-        <v>0.579104</v>
+        <v>0.6210830000000001</v>
       </c>
       <c r="N7" t="n">
         <v>0.2</v>
@@ -1141,7 +1133,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732034_12.txt</t>
+          <t>_2_12_1_1790732034_18.txt</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
@@ -1171,35 +1163,43 @@
         <v>0.1</v>
       </c>
       <c r="B8" t="n">
-        <v>0.239179</v>
+        <v>0.182872</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1790732086</v>
+        <v>1790732034</v>
       </c>
       <c r="E8" t="n">
-        <v>170</v>
+        <v>52</v>
       </c>
       <c r="F8" t="n">
         <v>200000</v>
       </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="n">
+        <v>0.586014</v>
+      </c>
       <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="inlineStr"/>
+        <v>0.65674</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.619364</v>
+      </c>
       <c r="J8" t="n">
-        <v>0.244267</v>
-      </c>
-      <c r="K8" t="inlineStr"/>
+        <v>0.183051</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.585635</v>
+      </c>
       <c r="L8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" t="inlineStr"/>
+        <v>0.623529</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.603989</v>
+      </c>
       <c r="N8" t="n">
         <v>0.2</v>
       </c>
@@ -1234,23 +1234,23 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732086_12.txt</t>
+          <t>_2_12_1_1790732034_0.txt</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z8" t="n">
         <v>12</v>
       </c>
       <c r="AA8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC8" t="inlineStr">
@@ -1264,7 +1264,7 @@
         <v>0.1</v>
       </c>
       <c r="B9" t="n">
-        <v>0.183464</v>
+        <v>0.185373</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1281,25 +1281,25 @@
         <v>200000</v>
       </c>
       <c r="G9" t="n">
-        <v>0.591382</v>
+        <v>0.557559</v>
       </c>
       <c r="H9" t="n">
-        <v>0.623824</v>
+        <v>0.630094</v>
       </c>
       <c r="I9" t="n">
-        <v>0.60717</v>
+        <v>0.591611</v>
       </c>
       <c r="J9" t="n">
-        <v>0.183931</v>
+        <v>0.183435</v>
       </c>
       <c r="K9" t="n">
-        <v>0.588571</v>
+        <v>0.584699</v>
       </c>
       <c r="L9" t="n">
-        <v>0.605882</v>
+        <v>0.629412</v>
       </c>
       <c r="M9" t="n">
-        <v>0.597102</v>
+        <v>0.606232</v>
       </c>
       <c r="N9" t="n">
         <v>0.2</v>
@@ -1335,7 +1335,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732034_7.txt</t>
+          <t>_2_12_1_1790732034_17.txt</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
@@ -1365,43 +1365,35 @@
         <v>0.1</v>
       </c>
       <c r="B10" t="n">
-        <v>0.182872</v>
+        <v>0.239731</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1790732034</v>
+        <v>1790732086</v>
       </c>
       <c r="E10" t="n">
-        <v>52</v>
+        <v>170</v>
       </c>
       <c r="F10" t="n">
         <v>200000</v>
       </c>
-      <c r="G10" t="n">
-        <v>0.586014</v>
-      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>0.65674</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0.619364</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" t="n">
-        <v>0.183051</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0.585635</v>
-      </c>
+        <v>0.245041</v>
+      </c>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="n">
-        <v>0.623529</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0.603989</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
         <v>0.2</v>
       </c>
@@ -1436,23 +1428,23 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732034_0.txt</t>
+          <t>_2_3_3_3_3_1_1790732086_15.txt</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z10" t="n">
         <v>12</v>
       </c>
       <c r="AA10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC10" t="inlineStr">
@@ -1466,7 +1458,7 @@
         <v>0.1</v>
       </c>
       <c r="B11" t="n">
-        <v>0.239077</v>
+        <v>0.239162</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1488,7 +1480,7 @@
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="n">
-        <v>0.244039</v>
+        <v>0.244353</v>
       </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
@@ -1529,7 +1521,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732086_2.txt</t>
+          <t>_2_3_3_3_3_1_1790732086_11.txt</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
@@ -1559,35 +1551,43 @@
         <v>0.1</v>
       </c>
       <c r="B12" t="n">
-        <v>0.239543</v>
+        <v>0.18729</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1790732086</v>
+        <v>1790732034</v>
       </c>
       <c r="E12" t="n">
-        <v>170</v>
+        <v>52</v>
       </c>
       <c r="F12" t="n">
         <v>200000</v>
       </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" t="n">
+        <v>0.593705</v>
+      </c>
       <c r="H12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" t="inlineStr"/>
+        <v>0.65047</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.620793</v>
+      </c>
       <c r="J12" t="n">
-        <v>0.244927</v>
-      </c>
-      <c r="K12" t="inlineStr"/>
+        <v>0.18561</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.6045199999999999</v>
+      </c>
       <c r="L12" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" t="inlineStr"/>
+        <v>0.629412</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.616715</v>
+      </c>
       <c r="N12" t="n">
         <v>0.2</v>
       </c>
@@ -1622,23 +1622,23 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732086_17.txt</t>
+          <t>_2_12_1_1790732034_10.txt</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z12" t="n">
         <v>12</v>
       </c>
       <c r="AA12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC12" t="inlineStr">
@@ -1652,43 +1652,35 @@
         <v>0.1</v>
       </c>
       <c r="B13" t="n">
-        <v>0.183899</v>
+        <v>0.239753</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1790732034</v>
+        <v>1790732086</v>
       </c>
       <c r="E13" t="n">
-        <v>52</v>
+        <v>170</v>
       </c>
       <c r="F13" t="n">
         <v>200000</v>
       </c>
-      <c r="G13" t="n">
-        <v>0.588571</v>
-      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>0.645768</v>
-      </c>
-      <c r="I13" t="n">
-        <v>0.615845</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I13" t="inlineStr"/>
       <c r="J13" t="n">
-        <v>0.183682</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0.606557</v>
-      </c>
+        <v>0.245059</v>
+      </c>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="n">
-        <v>0.652941</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0.628895</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M13" t="inlineStr"/>
       <c r="N13" t="n">
         <v>0.2</v>
       </c>
@@ -1723,23 +1715,23 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732034_1.txt</t>
+          <t>_2_3_3_3_3_1_1790732086_8.txt</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z13" t="n">
         <v>12</v>
       </c>
       <c r="AA13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
@@ -1753,7 +1745,7 @@
         <v>0.1</v>
       </c>
       <c r="B14" t="n">
-        <v>0.239741</v>
+        <v>0.23975</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1775,7 +1767,7 @@
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="n">
-        <v>0.24497</v>
+        <v>0.2451</v>
       </c>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="n">
@@ -1816,7 +1808,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732086_19.txt</t>
+          <t>_2_3_3_3_3_1_1790732086_5.txt</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
@@ -1846,35 +1838,43 @@
         <v>0.1</v>
       </c>
       <c r="B15" t="n">
-        <v>0.239729</v>
+        <v>0.1812</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1790732086</v>
+        <v>1790732034</v>
       </c>
       <c r="E15" t="n">
-        <v>170</v>
+        <v>52</v>
       </c>
       <c r="F15" t="n">
         <v>200000</v>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="n">
+        <v>0.572263</v>
+      </c>
       <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" t="inlineStr"/>
+        <v>0.61442</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.592593</v>
+      </c>
       <c r="J15" t="n">
-        <v>0.245052</v>
-      </c>
-      <c r="K15" t="inlineStr"/>
+        <v>0.180903</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.587209</v>
+      </c>
       <c r="L15" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" t="inlineStr"/>
+        <v>0.594118</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.590643</v>
+      </c>
       <c r="N15" t="n">
         <v>0.2</v>
       </c>
@@ -1909,23 +1909,23 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732086_6.txt</t>
+          <t>_2_12_1_1790732034_2.txt</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z15" t="n">
         <v>12</v>
       </c>
       <c r="AA15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
@@ -1939,35 +1939,43 @@
         <v>0.1</v>
       </c>
       <c r="B16" t="n">
-        <v>0.239693</v>
+        <v>0.180237</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1790732086</v>
+        <v>1790732034</v>
       </c>
       <c r="E16" t="n">
-        <v>170</v>
+        <v>52</v>
       </c>
       <c r="F16" t="n">
         <v>200000</v>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="n">
+        <v>0.587808</v>
+      </c>
       <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" t="inlineStr"/>
+        <v>0.634796</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.610399</v>
+      </c>
       <c r="J16" t="n">
-        <v>0.244958</v>
-      </c>
-      <c r="K16" t="inlineStr"/>
+        <v>0.182301</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.5705519999999999</v>
+      </c>
       <c r="L16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" t="inlineStr"/>
+        <v>0.547059</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.558559</v>
+      </c>
       <c r="N16" t="n">
         <v>0.2</v>
       </c>
@@ -2002,23 +2010,23 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732086_0.txt</t>
+          <t>_2_12_1_1790732034_19.txt</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z16" t="n">
         <v>12</v>
       </c>
       <c r="AA16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC16" t="inlineStr">
@@ -2032,43 +2040,35 @@
         <v>0.1</v>
       </c>
       <c r="B17" t="n">
-        <v>0.179732</v>
+        <v>0.239747</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1790732034</v>
+        <v>1790732086</v>
       </c>
       <c r="E17" t="n">
-        <v>52</v>
+        <v>170</v>
       </c>
       <c r="F17" t="n">
         <v>200000</v>
       </c>
-      <c r="G17" t="n">
-        <v>0.592958</v>
-      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>0.659875</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0.624629</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I17" t="inlineStr"/>
       <c r="J17" t="n">
-        <v>0.183519</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0.578947</v>
-      </c>
+        <v>0.245023</v>
+      </c>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="n">
-        <v>0.582353</v>
-      </c>
-      <c r="M17" t="n">
-        <v>0.580645</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M17" t="inlineStr"/>
       <c r="N17" t="n">
         <v>0.2</v>
       </c>
@@ -2103,23 +2103,23 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732034_11.txt</t>
+          <t>_2_3_3_3_3_1_1790732086_10.txt</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z17" t="n">
         <v>12</v>
       </c>
       <c r="AA17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC17" t="inlineStr">
@@ -2133,43 +2133,35 @@
         <v>0.1</v>
       </c>
       <c r="B18" t="n">
-        <v>0.180237</v>
+        <v>0.239744</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1790732034</v>
+        <v>1790732086</v>
       </c>
       <c r="E18" t="n">
-        <v>52</v>
+        <v>170</v>
       </c>
       <c r="F18" t="n">
         <v>200000</v>
       </c>
-      <c r="G18" t="n">
-        <v>0.587808</v>
-      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>0.634796</v>
-      </c>
-      <c r="I18" t="n">
-        <v>0.610399</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I18" t="inlineStr"/>
       <c r="J18" t="n">
-        <v>0.182301</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0.5705519999999999</v>
-      </c>
+        <v>0.245048</v>
+      </c>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="n">
-        <v>0.547059</v>
-      </c>
-      <c r="M18" t="n">
-        <v>0.558559</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M18" t="inlineStr"/>
       <c r="N18" t="n">
         <v>0.2</v>
       </c>
@@ -2204,23 +2196,23 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732034_19.txt</t>
+          <t>_2_3_3_3_3_1_1790732086_1.txt</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z18" t="n">
         <v>12</v>
       </c>
       <c r="AA18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC18" t="inlineStr">
@@ -2234,43 +2226,35 @@
         <v>0.1</v>
       </c>
       <c r="B19" t="n">
-        <v>0.180228</v>
+        <v>0.239741</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1790732034</v>
+        <v>1790732086</v>
       </c>
       <c r="E19" t="n">
-        <v>52</v>
+        <v>170</v>
       </c>
       <c r="F19" t="n">
         <v>200000</v>
       </c>
-      <c r="G19" t="n">
-        <v>0.597615</v>
-      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>0.6285269999999999</v>
-      </c>
-      <c r="I19" t="n">
-        <v>0.612681</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I19" t="inlineStr"/>
       <c r="J19" t="n">
-        <v>0.179652</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0.6303029999999999</v>
-      </c>
+        <v>0.24497</v>
+      </c>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="n">
-        <v>0.611765</v>
-      </c>
-      <c r="M19" t="n">
-        <v>0.620896</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M19" t="inlineStr"/>
       <c r="N19" t="n">
         <v>0.2</v>
       </c>
@@ -2305,23 +2289,23 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732034_5.txt</t>
+          <t>_2_3_3_3_3_1_1790732086_19.txt</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z19" t="n">
         <v>12</v>
       </c>
       <c r="AA19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC19" t="inlineStr">
@@ -2335,35 +2319,43 @@
         <v>0.1</v>
       </c>
       <c r="B20" t="n">
-        <v>0.239162</v>
+        <v>0.178623</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1790732086</v>
+        <v>1790732034</v>
       </c>
       <c r="E20" t="n">
-        <v>170</v>
+        <v>52</v>
       </c>
       <c r="F20" t="n">
         <v>200000</v>
       </c>
-      <c r="G20" t="inlineStr"/>
+      <c r="G20" t="n">
+        <v>0.600293</v>
+      </c>
       <c r="H20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" t="inlineStr"/>
+        <v>0.642633</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.620742</v>
+      </c>
       <c r="J20" t="n">
-        <v>0.244353</v>
-      </c>
-      <c r="K20" t="inlineStr"/>
+        <v>0.181897</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0.616279</v>
+      </c>
       <c r="L20" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" t="inlineStr"/>
+        <v>0.623529</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0.619883</v>
+      </c>
       <c r="N20" t="n">
         <v>0.2</v>
       </c>
@@ -2398,23 +2390,23 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732086_11.txt</t>
+          <t>_2_12_1_1790732034_3.txt</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z20" t="n">
         <v>12</v>
       </c>
       <c r="AA20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC20" t="inlineStr">
@@ -2428,7 +2420,7 @@
         <v>0.1</v>
       </c>
       <c r="B21" t="n">
-        <v>0.181265</v>
+        <v>0.175663</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2445,25 +2437,25 @@
         <v>200000</v>
       </c>
       <c r="G21" t="n">
-        <v>0.562323</v>
+        <v>0.616864</v>
       </c>
       <c r="H21" t="n">
-        <v>0.6222569999999999</v>
+        <v>0.653605</v>
       </c>
       <c r="I21" t="n">
-        <v>0.590774</v>
+        <v>0.634703</v>
       </c>
       <c r="J21" t="n">
-        <v>0.179788</v>
+        <v>0.17518</v>
       </c>
       <c r="K21" t="n">
-        <v>0.58011</v>
+        <v>0.631579</v>
       </c>
       <c r="L21" t="n">
-        <v>0.6176469999999999</v>
+        <v>0.635294</v>
       </c>
       <c r="M21" t="n">
-        <v>0.598291</v>
+        <v>0.633431</v>
       </c>
       <c r="N21" t="n">
         <v>0.2</v>
@@ -2499,7 +2491,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732034_8.txt</t>
+          <t>_2_12_1_1790732034_6.txt</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
@@ -2529,7 +2521,7 @@
         <v>0.1</v>
       </c>
       <c r="B22" t="n">
-        <v>0.1812</v>
+        <v>0.181265</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -2546,25 +2538,25 @@
         <v>200000</v>
       </c>
       <c r="G22" t="n">
-        <v>0.572263</v>
+        <v>0.562323</v>
       </c>
       <c r="H22" t="n">
-        <v>0.61442</v>
+        <v>0.6222569999999999</v>
       </c>
       <c r="I22" t="n">
-        <v>0.592593</v>
+        <v>0.590774</v>
       </c>
       <c r="J22" t="n">
-        <v>0.180903</v>
+        <v>0.179788</v>
       </c>
       <c r="K22" t="n">
-        <v>0.587209</v>
+        <v>0.58011</v>
       </c>
       <c r="L22" t="n">
-        <v>0.594118</v>
+        <v>0.6176469999999999</v>
       </c>
       <c r="M22" t="n">
-        <v>0.590643</v>
+        <v>0.598291</v>
       </c>
       <c r="N22" t="n">
         <v>0.2</v>
@@ -2600,7 +2592,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732034_2.txt</t>
+          <t>_2_12_1_1790732034_8.txt</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
@@ -2723,7 +2715,7 @@
         <v>0.1</v>
       </c>
       <c r="B24" t="n">
-        <v>0.239735</v>
+        <v>0.239179</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2745,7 +2737,7 @@
       </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="n">
-        <v>0.24501</v>
+        <v>0.244267</v>
       </c>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="n">
@@ -2786,7 +2778,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732086_7.txt</t>
+          <t>_2_3_3_3_3_1_1790732086_12.txt</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
@@ -2816,7 +2808,7 @@
         <v>0.1</v>
       </c>
       <c r="B25" t="n">
-        <v>0.239753</v>
+        <v>0.236779</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2838,7 +2830,7 @@
       </c>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="n">
-        <v>0.245059</v>
+        <v>0.242342</v>
       </c>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="n">
@@ -2879,7 +2871,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732086_8.txt</t>
+          <t>_2_3_3_3_3_1_1790732086_9.txt</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
@@ -2909,7 +2901,7 @@
         <v>0.1</v>
       </c>
       <c r="B26" t="n">
-        <v>0.239744</v>
+        <v>0.239609</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -2931,7 +2923,7 @@
       </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="n">
-        <v>0.245048</v>
+        <v>0.244874</v>
       </c>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="n">
@@ -2972,7 +2964,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732086_1.txt</t>
+          <t>_2_3_3_3_3_1_1790732086_4.txt</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
@@ -3002,43 +2994,35 @@
         <v>0.1</v>
       </c>
       <c r="B27" t="n">
-        <v>0.185877</v>
+        <v>0.239749</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1790732034</v>
+        <v>1790732086</v>
       </c>
       <c r="E27" t="n">
-        <v>52</v>
+        <v>170</v>
       </c>
       <c r="F27" t="n">
         <v>200000</v>
       </c>
-      <c r="G27" t="n">
-        <v>0.576052</v>
-      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>0.557994</v>
-      </c>
-      <c r="I27" t="n">
-        <v>0.566879</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I27" t="inlineStr"/>
       <c r="J27" t="n">
-        <v>0.185751</v>
-      </c>
-      <c r="K27" t="n">
-        <v>0.582192</v>
-      </c>
+        <v>0.245062</v>
+      </c>
+      <c r="K27" t="inlineStr"/>
       <c r="L27" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="M27" t="n">
-        <v>0.537975</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M27" t="inlineStr"/>
       <c r="N27" t="n">
         <v>0.2</v>
       </c>
@@ -3073,23 +3057,23 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732034_14.txt</t>
+          <t>_2_3_3_3_3_1_1790732086_18.txt</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z27" t="n">
         <v>12</v>
       </c>
       <c r="AA27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB27" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC27" t="inlineStr">
@@ -3103,43 +3087,35 @@
         <v>0.1</v>
       </c>
       <c r="B28" t="n">
-        <v>0.183868</v>
+        <v>0.239748</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1790732034</v>
+        <v>1790732086</v>
       </c>
       <c r="E28" t="n">
-        <v>52</v>
+        <v>170</v>
       </c>
       <c r="F28" t="n">
         <v>200000</v>
       </c>
-      <c r="G28" t="n">
-        <v>0.5686</v>
-      </c>
+      <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>0.630094</v>
-      </c>
-      <c r="I28" t="n">
-        <v>0.59777</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I28" t="inlineStr"/>
       <c r="J28" t="n">
-        <v>0.18723</v>
-      </c>
-      <c r="K28" t="n">
-        <v>0.5672509999999999</v>
-      </c>
+        <v>0.245065</v>
+      </c>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" t="n">
-        <v>0.570588</v>
-      </c>
-      <c r="M28" t="n">
-        <v>0.5689149999999999</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M28" t="inlineStr"/>
       <c r="N28" t="n">
         <v>0.2</v>
       </c>
@@ -3174,23 +3150,23 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732034_9.txt</t>
+          <t>_2_3_3_3_3_1_1790732086_3.txt</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z28" t="n">
         <v>12</v>
       </c>
       <c r="AA28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB28" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC28" t="inlineStr">
@@ -3204,35 +3180,43 @@
         <v>0.1</v>
       </c>
       <c r="B29" t="n">
-        <v>0.239731</v>
+        <v>0.183899</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1790732086</v>
+        <v>1790732034</v>
       </c>
       <c r="E29" t="n">
-        <v>170</v>
+        <v>52</v>
       </c>
       <c r="F29" t="n">
         <v>200000</v>
       </c>
-      <c r="G29" t="inlineStr"/>
+      <c r="G29" t="n">
+        <v>0.588571</v>
+      </c>
       <c r="H29" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" t="inlineStr"/>
+        <v>0.645768</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.615845</v>
+      </c>
       <c r="J29" t="n">
-        <v>0.245041</v>
-      </c>
-      <c r="K29" t="inlineStr"/>
+        <v>0.183682</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0.606557</v>
+      </c>
       <c r="L29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M29" t="inlineStr"/>
+        <v>0.652941</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0.628895</v>
+      </c>
       <c r="N29" t="n">
         <v>0.2</v>
       </c>
@@ -3267,23 +3251,23 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732086_15.txt</t>
+          <t>_2_12_1_1790732034_1.txt</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z29" t="n">
         <v>12</v>
       </c>
       <c r="AA29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB29" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC29" t="inlineStr">
@@ -3297,43 +3281,35 @@
         <v>0.1</v>
       </c>
       <c r="B30" t="n">
-        <v>0.178602</v>
+        <v>0.239077</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1790732034</v>
+        <v>1790732086</v>
       </c>
       <c r="E30" t="n">
-        <v>52</v>
+        <v>170</v>
       </c>
       <c r="F30" t="n">
         <v>200000</v>
       </c>
-      <c r="G30" t="n">
-        <v>0.600299</v>
-      </c>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>0.6285269999999999</v>
-      </c>
-      <c r="I30" t="n">
-        <v>0.614089</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I30" t="inlineStr"/>
       <c r="J30" t="n">
-        <v>0.178801</v>
-      </c>
-      <c r="K30" t="n">
-        <v>0.601156</v>
-      </c>
+        <v>0.244039</v>
+      </c>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="n">
-        <v>0.611765</v>
-      </c>
-      <c r="M30" t="n">
-        <v>0.606414</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M30" t="inlineStr"/>
       <c r="N30" t="n">
         <v>0.2</v>
       </c>
@@ -3368,23 +3344,23 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732034_13.txt</t>
+          <t>_2_3_3_3_3_1_1790732086_2.txt</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z30" t="n">
         <v>12</v>
       </c>
       <c r="AA30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB30" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC30" t="inlineStr">
@@ -3398,35 +3374,43 @@
         <v>0.1</v>
       </c>
       <c r="B31" t="n">
-        <v>0.239609</v>
+        <v>0.173092</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1790732086</v>
+        <v>1790732034</v>
       </c>
       <c r="E31" t="n">
-        <v>170</v>
+        <v>52</v>
       </c>
       <c r="F31" t="n">
         <v>200000</v>
       </c>
-      <c r="G31" t="inlineStr"/>
+      <c r="G31" t="n">
+        <v>0.628319</v>
+      </c>
       <c r="H31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" t="inlineStr"/>
+        <v>0.667712</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.647416</v>
+      </c>
       <c r="J31" t="n">
-        <v>0.244874</v>
-      </c>
-      <c r="K31" t="inlineStr"/>
+        <v>0.173815</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0.594118</v>
+      </c>
       <c r="L31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M31" t="inlineStr"/>
+        <v>0.594118</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0.594118</v>
+      </c>
       <c r="N31" t="n">
         <v>0.2</v>
       </c>
@@ -3461,23 +3445,23 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732086_4.txt</t>
+          <t>_2_12_1_1790732034_15.txt</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z31" t="n">
         <v>12</v>
       </c>
       <c r="AA31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC31" t="inlineStr">
@@ -3491,35 +3475,43 @@
         <v>0.1</v>
       </c>
       <c r="B32" t="n">
-        <v>0.239748</v>
+        <v>0.183464</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1790732086</v>
+        <v>1790732034</v>
       </c>
       <c r="E32" t="n">
-        <v>170</v>
+        <v>52</v>
       </c>
       <c r="F32" t="n">
         <v>200000</v>
       </c>
-      <c r="G32" t="inlineStr"/>
+      <c r="G32" t="n">
+        <v>0.591382</v>
+      </c>
       <c r="H32" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" t="inlineStr"/>
+        <v>0.623824</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.60717</v>
+      </c>
       <c r="J32" t="n">
-        <v>0.245065</v>
-      </c>
-      <c r="K32" t="inlineStr"/>
+        <v>0.183931</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0.588571</v>
+      </c>
       <c r="L32" t="n">
-        <v>0</v>
-      </c>
-      <c r="M32" t="inlineStr"/>
+        <v>0.605882</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0.597102</v>
+      </c>
       <c r="N32" t="n">
         <v>0.2</v>
       </c>
@@ -3554,23 +3546,23 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732086_3.txt</t>
+          <t>_2_12_1_1790732034_7.txt</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z32" t="n">
         <v>12</v>
       </c>
       <c r="AA32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC32" t="inlineStr">
@@ -3584,43 +3576,35 @@
         <v>0.1</v>
       </c>
       <c r="B33" t="n">
-        <v>0.183638</v>
+        <v>0.239733</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1790732034</v>
+        <v>1790732086</v>
       </c>
       <c r="E33" t="n">
-        <v>52</v>
+        <v>170</v>
       </c>
       <c r="F33" t="n">
         <v>200000</v>
       </c>
-      <c r="G33" t="n">
-        <v>0.5625</v>
-      </c>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>0.648903</v>
-      </c>
-      <c r="I33" t="n">
-        <v>0.60262</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I33" t="inlineStr"/>
       <c r="J33" t="n">
-        <v>0.180978</v>
-      </c>
-      <c r="K33" t="n">
-        <v>0.590164</v>
-      </c>
+        <v>0.245114</v>
+      </c>
+      <c r="K33" t="inlineStr"/>
       <c r="L33" t="n">
-        <v>0.635294</v>
-      </c>
-      <c r="M33" t="n">
-        <v>0.6118980000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M33" t="inlineStr"/>
       <c r="N33" t="n">
         <v>0.2</v>
       </c>
@@ -3655,23 +3639,23 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732034_4.txt</t>
+          <t>_2_3_3_3_3_1_1790732086_16.txt</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z33" t="n">
         <v>12</v>
       </c>
       <c r="AA33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB33" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC33" t="inlineStr">
@@ -3685,7 +3669,7 @@
         <v>0.1</v>
       </c>
       <c r="B34" t="n">
-        <v>0.185373</v>
+        <v>0.179732</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -3702,25 +3686,25 @@
         <v>200000</v>
       </c>
       <c r="G34" t="n">
-        <v>0.557559</v>
+        <v>0.592958</v>
       </c>
       <c r="H34" t="n">
-        <v>0.630094</v>
+        <v>0.659875</v>
       </c>
       <c r="I34" t="n">
-        <v>0.591611</v>
+        <v>0.624629</v>
       </c>
       <c r="J34" t="n">
-        <v>0.183435</v>
+        <v>0.183519</v>
       </c>
       <c r="K34" t="n">
-        <v>0.584699</v>
+        <v>0.578947</v>
       </c>
       <c r="L34" t="n">
-        <v>0.629412</v>
+        <v>0.582353</v>
       </c>
       <c r="M34" t="n">
-        <v>0.606232</v>
+        <v>0.580645</v>
       </c>
       <c r="N34" t="n">
         <v>0.2</v>
@@ -3756,7 +3740,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732034_17.txt</t>
+          <t>_2_12_1_1790732034_11.txt</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
@@ -3786,7 +3770,7 @@
         <v>0.1</v>
       </c>
       <c r="B35" t="n">
-        <v>0.173092</v>
+        <v>0.183868</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -3803,25 +3787,25 @@
         <v>200000</v>
       </c>
       <c r="G35" t="n">
-        <v>0.628319</v>
+        <v>0.5686</v>
       </c>
       <c r="H35" t="n">
-        <v>0.667712</v>
+        <v>0.630094</v>
       </c>
       <c r="I35" t="n">
-        <v>0.647416</v>
+        <v>0.59777</v>
       </c>
       <c r="J35" t="n">
-        <v>0.173815</v>
+        <v>0.18723</v>
       </c>
       <c r="K35" t="n">
-        <v>0.594118</v>
+        <v>0.5672509999999999</v>
       </c>
       <c r="L35" t="n">
-        <v>0.594118</v>
+        <v>0.570588</v>
       </c>
       <c r="M35" t="n">
-        <v>0.594118</v>
+        <v>0.5689149999999999</v>
       </c>
       <c r="N35" t="n">
         <v>0.2</v>
@@ -3857,7 +3841,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732034_15.txt</t>
+          <t>_2_12_1_1790732034_9.txt</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
@@ -3887,7 +3871,7 @@
         <v>0.1</v>
       </c>
       <c r="B36" t="n">
-        <v>0.18729</v>
+        <v>0.185877</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -3904,25 +3888,25 @@
         <v>200000</v>
       </c>
       <c r="G36" t="n">
-        <v>0.593705</v>
+        <v>0.576052</v>
       </c>
       <c r="H36" t="n">
-        <v>0.65047</v>
+        <v>0.557994</v>
       </c>
       <c r="I36" t="n">
-        <v>0.620793</v>
+        <v>0.566879</v>
       </c>
       <c r="J36" t="n">
-        <v>0.18561</v>
+        <v>0.185751</v>
       </c>
       <c r="K36" t="n">
-        <v>0.6045199999999999</v>
+        <v>0.582192</v>
       </c>
       <c r="L36" t="n">
-        <v>0.629412</v>
+        <v>0.5</v>
       </c>
       <c r="M36" t="n">
-        <v>0.616715</v>
+        <v>0.537975</v>
       </c>
       <c r="N36" t="n">
         <v>0.2</v>
@@ -3958,7 +3942,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732034_10.txt</t>
+          <t>_2_12_1_1790732034_14.txt</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
@@ -3988,35 +3972,43 @@
         <v>0.1</v>
       </c>
       <c r="B37" t="n">
-        <v>0.239733</v>
+        <v>0.178602</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1790732086</v>
+        <v>1790732034</v>
       </c>
       <c r="E37" t="n">
-        <v>170</v>
+        <v>52</v>
       </c>
       <c r="F37" t="n">
         <v>200000</v>
       </c>
-      <c r="G37" t="inlineStr"/>
+      <c r="G37" t="n">
+        <v>0.600299</v>
+      </c>
       <c r="H37" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" t="inlineStr"/>
+        <v>0.6285269999999999</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.614089</v>
+      </c>
       <c r="J37" t="n">
-        <v>0.245085</v>
-      </c>
-      <c r="K37" t="inlineStr"/>
+        <v>0.178801</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0.601156</v>
+      </c>
       <c r="L37" t="n">
-        <v>0</v>
-      </c>
-      <c r="M37" t="inlineStr"/>
+        <v>0.611765</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0.606414</v>
+      </c>
       <c r="N37" t="n">
         <v>0.2</v>
       </c>
@@ -4051,23 +4043,23 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732086_14.txt</t>
+          <t>_2_12_1_1790732034_13.txt</t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z37" t="n">
         <v>12</v>
       </c>
       <c r="AA37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB37" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC37" t="inlineStr">
@@ -4081,7 +4073,7 @@
         <v>0.1</v>
       </c>
       <c r="B38" t="n">
-        <v>0.239733</v>
+        <v>0.239543</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -4103,7 +4095,7 @@
       </c>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="n">
-        <v>0.245114</v>
+        <v>0.244927</v>
       </c>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="n">
@@ -4144,7 +4136,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732086_16.txt</t>
+          <t>_2_3_3_3_3_1_1790732086_17.txt</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
@@ -4174,7 +4166,7 @@
         <v>0.1</v>
       </c>
       <c r="B39" t="n">
-        <v>0.184394</v>
+        <v>0.180228</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -4191,25 +4183,25 @@
         <v>200000</v>
       </c>
       <c r="G39" t="n">
-        <v>0.610015</v>
+        <v>0.597615</v>
       </c>
       <c r="H39" t="n">
-        <v>0.630094</v>
+        <v>0.6285269999999999</v>
       </c>
       <c r="I39" t="n">
-        <v>0.619892</v>
+        <v>0.612681</v>
       </c>
       <c r="J39" t="n">
-        <v>0.184358</v>
+        <v>0.179652</v>
       </c>
       <c r="K39" t="n">
-        <v>0.614907</v>
+        <v>0.6303029999999999</v>
       </c>
       <c r="L39" t="n">
-        <v>0.582353</v>
+        <v>0.611765</v>
       </c>
       <c r="M39" t="n">
-        <v>0.598187</v>
+        <v>0.620896</v>
       </c>
       <c r="N39" t="n">
         <v>0.2</v>
@@ -4245,7 +4237,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732034_16.txt</t>
+          <t>_2_12_1_1790732034_5.txt</t>
         </is>
       </c>
       <c r="Y39" t="inlineStr">
@@ -4275,35 +4267,43 @@
         <v>0.1</v>
       </c>
       <c r="B40" t="n">
-        <v>0.239749</v>
+        <v>0.180623</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>1790732086</v>
+        <v>1790732034</v>
       </c>
       <c r="E40" t="n">
-        <v>170</v>
+        <v>52</v>
       </c>
       <c r="F40" t="n">
         <v>200000</v>
       </c>
-      <c r="G40" t="inlineStr"/>
+      <c r="G40" t="n">
+        <v>0.583573</v>
+      </c>
       <c r="H40" t="n">
-        <v>0</v>
-      </c>
-      <c r="I40" t="inlineStr"/>
+        <v>0.634796</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0.608108</v>
+      </c>
       <c r="J40" t="n">
-        <v>0.245062</v>
-      </c>
-      <c r="K40" t="inlineStr"/>
+        <v>0.180828</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0.587879</v>
+      </c>
       <c r="L40" t="n">
-        <v>0</v>
-      </c>
-      <c r="M40" t="inlineStr"/>
+        <v>0.570588</v>
+      </c>
+      <c r="M40" t="n">
+        <v>0.579104</v>
+      </c>
       <c r="N40" t="n">
         <v>0.2</v>
       </c>
@@ -4338,23 +4338,23 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732086_18.txt</t>
+          <t>_2_12_1_1790732034_12.txt</t>
         </is>
       </c>
       <c r="Y40" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z40" t="n">
         <v>12</v>
       </c>
       <c r="AA40" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB40" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC40" t="inlineStr">
@@ -4368,7 +4368,7 @@
         <v>0.1</v>
       </c>
       <c r="B41" t="n">
-        <v>0.23975</v>
+        <v>0.239729</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -4390,7 +4390,7 @@
       </c>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="n">
-        <v>0.2451</v>
+        <v>0.245052</v>
       </c>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="n">
@@ -4431,7 +4431,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732086_5.txt</t>
+          <t>_2_3_3_3_3_1_1790732086_6.txt</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr">
@@ -4522,7 +4522,7 @@
         <v>0.59864875</v>
       </c>
       <c r="C2" t="n">
-        <v>0.02426617552517128</v>
+        <v>0.02426617552517125</v>
       </c>
       <c r="D2" t="n">
         <v>0.633431</v>

</xml_diff>